<commit_message>
feat: kolom Jabatan di Excel mencalonkan penghuni kursi kosong
Kolom baru (WARGA/DUKUH/RW/RT) dibaca HANYA untuk kursi yang masih kosong.
Begitu kursinya terisi, kolom itu diabaikan — kalau tidak, satu impor Excel
yang belum diperbarui bisa membatalkan pergantian yang sudah disetujui Dukuh
dan para Ketua RW. Kolom ini bukan penentu kewenangan; yang menentukan tetap
akun di tabel pengurus.

Dua orang ditandai memegang kursi yang sama menghentikan impor sebelum satu
baris pun ditulis.

docs/data-penduduk.xlsx diisi 1 Dukuh + 3 RW + 6 RT (kepala keluarga tertua di
tiap wilayah) dan 375 warga.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data-penduduk.xlsx
+++ b/docs/data-penduduk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Data Penduduk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data Penduduk'!$A$2:$T$387</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data Penduduk'!$A$2:$U$387</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T387"/>
+  <dimension ref="A1:U387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -480,6 +480,7 @@
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1"/>
@@ -584,6 +585,11 @@
           <t>Kode Pos</t>
         </is>
       </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>Jabatan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -686,6 +692,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U3" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -788,6 +799,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -890,6 +906,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -992,6 +1013,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U6" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1094,6 +1120,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1196,6 +1227,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1298,6 +1334,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1400,6 +1441,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U10" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1502,6 +1548,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U11" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1604,6 +1655,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U12" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1706,6 +1762,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1808,6 +1869,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U14" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1910,6 +1976,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -2012,6 +2083,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U16" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -2114,6 +2190,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>DUKUH</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -2216,6 +2297,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -2318,6 +2404,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -2420,6 +2511,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U20" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2522,6 +2618,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2624,6 +2725,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2726,6 +2832,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2828,6 +2939,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U24" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2930,6 +3046,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -3032,6 +3153,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -3134,6 +3260,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -3236,6 +3367,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U28" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -3338,6 +3474,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -3440,6 +3581,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -3542,6 +3688,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -3644,6 +3795,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U32" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -3746,6 +3902,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -3848,6 +4009,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U34" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -3950,6 +4116,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -4052,6 +4223,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U36" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -4154,6 +4330,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -4256,6 +4437,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -4358,6 +4544,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -4460,6 +4651,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U40" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -4562,6 +4758,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -4664,6 +4865,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U42" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -4766,6 +4972,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U43" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -4868,6 +5079,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U44" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -4970,6 +5186,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U45" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -5072,6 +5293,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U46" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -5174,6 +5400,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U47" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -5276,6 +5507,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U48" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -5378,6 +5614,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U49" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -5480,6 +5721,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U50" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -5582,6 +5828,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U51" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -5684,6 +5935,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U52" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -5786,6 +6042,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U53" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -5888,6 +6149,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U54" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -5990,6 +6256,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U55" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -6092,6 +6363,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U56" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -6194,6 +6470,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U57" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -6296,6 +6577,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U58" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -6398,6 +6684,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U59" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -6500,6 +6791,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U60" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -6602,6 +6898,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U61" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -6704,6 +7005,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U62" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -6806,6 +7112,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U63" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -6908,6 +7219,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U64" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -7010,6 +7326,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U65" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -7112,6 +7433,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U66" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -7214,6 +7540,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U67" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -7316,6 +7647,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U68" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -7418,6 +7754,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U69" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -7520,6 +7861,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U70" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -7622,6 +7968,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U71" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -7724,6 +8075,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U72" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -7826,6 +8182,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U73" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -7928,6 +8289,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U74" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -8030,6 +8396,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U75" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -8132,6 +8503,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U76" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -8234,6 +8610,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U77" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -8336,6 +8717,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U78" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -8438,6 +8824,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U79" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -8540,6 +8931,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U80" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -8642,6 +9038,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U81" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -8744,6 +9145,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U82" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -8846,6 +9252,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U83" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -8948,6 +9359,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U84" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -9050,6 +9466,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U85" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -9152,6 +9573,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U86" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -9254,6 +9680,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U87" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -9356,6 +9787,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U88" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -9458,6 +9894,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U89" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -9560,6 +10001,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U90" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -9662,6 +10108,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U91" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -9764,6 +10215,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U92" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -9866,6 +10322,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U93" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -9968,6 +10429,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U94" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -10070,6 +10536,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U95" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -10172,6 +10643,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U96" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -10274,6 +10750,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U97" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -10376,6 +10857,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U98" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -10478,6 +10964,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U99" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -10580,6 +11071,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U100" s="4" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -10682,6 +11178,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U101" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -10784,6 +11285,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U102" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -10886,6 +11392,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U103" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -10988,6 +11499,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U104" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -11090,6 +11606,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U105" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -11192,6 +11713,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U106" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -11294,6 +11820,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U107" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -11396,6 +11927,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U108" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -11498,6 +12034,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U109" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -11600,6 +12141,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U110" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -11702,6 +12248,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U111" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -11804,6 +12355,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U112" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -11906,6 +12462,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U113" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
@@ -12008,6 +12569,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U114" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -12110,6 +12676,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U115" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
@@ -12212,6 +12783,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U116" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -12314,6 +12890,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U117" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -12416,6 +12997,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U118" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -12518,6 +13104,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U119" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
@@ -12620,6 +13211,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U120" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -12722,6 +13318,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U121" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
@@ -12824,6 +13425,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U122" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -12926,6 +13532,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U123" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -13028,6 +13639,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U124" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -13130,6 +13746,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U125" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -13232,6 +13853,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U126" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -13334,6 +13960,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U127" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -13436,6 +14067,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U128" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -13538,6 +14174,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U129" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
@@ -13640,6 +14281,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U130" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -13742,6 +14388,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U131" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
@@ -13844,6 +14495,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U132" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -13946,6 +14602,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U133" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
@@ -14048,6 +14709,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U134" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -14150,6 +14816,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U135" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -14252,6 +14923,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U136" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -14354,6 +15030,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U137" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
@@ -14456,6 +15137,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U138" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -14558,6 +15244,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U139" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -14660,6 +15351,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U140" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -14762,6 +15458,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U141" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -14864,6 +15565,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U142" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -14966,6 +15672,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U143" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
@@ -15068,6 +15779,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U144" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -15170,6 +15886,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U145" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -15272,6 +15993,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U146" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -15374,6 +16100,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U147" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
@@ -15476,6 +16207,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U148" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -15578,6 +16314,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U149" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -15680,6 +16421,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U150" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -15782,6 +16528,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U151" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
@@ -15884,6 +16635,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U152" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -15986,6 +16742,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U153" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -16088,6 +16849,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U154" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -16190,6 +16956,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U155" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -16292,6 +17063,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U156" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -16394,6 +17170,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U157" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -16496,6 +17277,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U158" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -16598,6 +17384,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U159" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -16700,6 +17491,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U160" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -16802,6 +17598,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U161" s="4" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -16904,6 +17705,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U162" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -17006,6 +17812,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U163" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -17108,6 +17919,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U164" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -17210,6 +18026,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U165" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -17312,6 +18133,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U166" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -17414,6 +18240,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U167" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
@@ -17516,6 +18347,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U168" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -17618,6 +18454,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U169" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -17720,6 +18561,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U170" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -17822,6 +18668,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U171" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -17924,6 +18775,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U172" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -18026,6 +18882,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U173" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -18128,6 +18989,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U174" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -18230,6 +19096,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U175" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
@@ -18332,6 +19203,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U176" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -18434,6 +19310,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U177" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
@@ -18536,6 +19417,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U178" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -18638,6 +19524,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U179" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
@@ -18740,6 +19631,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U180" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -18842,6 +19738,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U181" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
@@ -18944,6 +19845,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U182" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
@@ -19046,6 +19952,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U183" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
@@ -19148,6 +20059,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U184" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
@@ -19250,6 +20166,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U185" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
@@ -19352,6 +20273,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U186" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -19454,6 +20380,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U187" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
@@ -19556,6 +20487,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U188" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
@@ -19658,6 +20594,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U189" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
@@ -19760,6 +20701,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U190" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
@@ -19862,6 +20808,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U191" s="4" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
@@ -19964,6 +20915,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U192" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
@@ -20066,6 +21022,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U193" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
@@ -20168,6 +21129,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U194" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
@@ -20270,6 +21236,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U195" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
@@ -20372,6 +21343,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U196" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
@@ -20474,6 +21450,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U197" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
@@ -20576,6 +21557,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U198" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
@@ -20678,6 +21664,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U199" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
@@ -20780,6 +21771,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U200" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
@@ -20882,6 +21878,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U201" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
@@ -20984,6 +21985,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U202" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
@@ -21086,6 +22092,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U203" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
@@ -21188,6 +22199,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U204" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
@@ -21290,6 +22306,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U205" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
@@ -21392,6 +22413,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U206" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
@@ -21494,6 +22520,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U207" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
@@ -21596,6 +22627,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U208" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
@@ -21698,6 +22734,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U209" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
@@ -21800,6 +22841,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U210" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
@@ -21902,6 +22948,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U211" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
@@ -22004,6 +23055,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U212" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
@@ -22106,6 +23162,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U213" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
@@ -22208,6 +23269,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U214" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
@@ -22310,6 +23376,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U215" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
@@ -22412,6 +23483,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U216" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
@@ -22514,6 +23590,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U217" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
@@ -22616,6 +23697,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U218" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
@@ -22718,6 +23804,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U219" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
@@ -22820,6 +23911,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U220" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
@@ -22922,6 +24018,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U221" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
@@ -23024,6 +24125,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U222" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
@@ -23126,6 +24232,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U223" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
@@ -23228,6 +24339,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U224" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
@@ -23330,6 +24446,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U225" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
@@ -23432,6 +24553,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U226" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
@@ -23534,6 +24660,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U227" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
@@ -23636,6 +24767,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U228" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
@@ -23738,6 +24874,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U229" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
@@ -23840,6 +24981,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U230" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
@@ -23942,6 +25088,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U231" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
@@ -24044,6 +25195,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U232" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
@@ -24146,6 +25302,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U233" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
@@ -24248,6 +25409,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U234" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
@@ -24350,6 +25516,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U235" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
@@ -24452,6 +25623,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U236" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
@@ -24554,6 +25730,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U237" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
@@ -24656,6 +25837,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U238" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
@@ -24758,6 +25944,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U239" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
@@ -24860,6 +26051,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U240" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
@@ -24962,6 +26158,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U241" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
@@ -25064,6 +26265,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U242" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
@@ -25166,6 +26372,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U243" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
@@ -25268,6 +26479,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U244" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
@@ -25370,6 +26586,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U245" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
@@ -25472,6 +26693,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U246" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
@@ -25574,6 +26800,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U247" s="4" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
@@ -25676,6 +26907,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U248" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
@@ -25778,6 +27014,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U249" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
@@ -25880,6 +27121,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U250" s="4" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
@@ -25982,6 +27228,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U251" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
@@ -26084,6 +27335,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U252" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
@@ -26186,6 +27442,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U253" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
@@ -26288,6 +27549,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U254" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
@@ -26390,6 +27656,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U255" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
@@ -26492,6 +27763,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U256" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
@@ -26594,6 +27870,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U257" s="4" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="4" t="inlineStr">
@@ -26696,6 +27977,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U258" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
@@ -26798,6 +28084,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U259" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
@@ -26900,6 +28191,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U260" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
@@ -27002,6 +28298,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U261" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="4" t="inlineStr">
@@ -27104,6 +28405,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U262" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
@@ -27206,6 +28512,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U263" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
@@ -27308,6 +28619,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U264" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
@@ -27410,6 +28726,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U265" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
@@ -27512,6 +28833,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U266" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
@@ -27614,6 +28940,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U267" s="4" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
@@ -27716,6 +29047,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U268" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
@@ -27818,6 +29154,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U269" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
@@ -27920,6 +29261,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U270" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
@@ -28022,6 +29368,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U271" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="4" t="inlineStr">
@@ -28124,6 +29475,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U272" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
@@ -28226,6 +29582,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U273" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
@@ -28328,6 +29689,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U274" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
@@ -28430,6 +29796,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U275" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="4" t="inlineStr">
@@ -28532,6 +29903,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U276" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
@@ -28634,6 +30010,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U277" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="4" t="inlineStr">
@@ -28736,6 +30117,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U278" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="4" t="inlineStr">
@@ -28838,6 +30224,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U279" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="4" t="inlineStr">
@@ -28940,6 +30331,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U280" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="4" t="inlineStr">
@@ -29042,6 +30438,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U281" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="4" t="inlineStr">
@@ -29144,6 +30545,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U282" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
@@ -29246,6 +30652,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U283" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="4" t="inlineStr">
@@ -29348,6 +30759,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U284" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
@@ -29450,6 +30866,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U285" s="4" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
@@ -29552,6 +30973,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U286" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
@@ -29654,6 +31080,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U287" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
@@ -29756,6 +31187,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U288" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
@@ -29858,6 +31294,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U289" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
@@ -29960,6 +31401,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U290" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
@@ -30062,6 +31508,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U291" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
@@ -30164,6 +31615,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U292" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
@@ -30266,6 +31722,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U293" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
@@ -30368,6 +31829,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U294" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
@@ -30470,6 +31936,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U295" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
@@ -30572,6 +32043,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U296" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
@@ -30674,6 +32150,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U297" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
@@ -30776,6 +32257,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U298" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
@@ -30878,6 +32364,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U299" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
@@ -30980,6 +32471,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U300" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
@@ -31082,6 +32578,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U301" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="4" t="inlineStr">
@@ -31184,6 +32685,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U302" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
@@ -31286,6 +32792,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U303" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
@@ -31388,6 +32899,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U304" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
@@ -31490,6 +33006,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U305" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="4" t="inlineStr">
@@ -31592,6 +33113,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U306" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
@@ -31694,6 +33220,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U307" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="4" t="inlineStr">
@@ -31796,6 +33327,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U308" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
@@ -31898,6 +33434,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U309" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="4" t="inlineStr">
@@ -32000,6 +33541,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U310" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
@@ -32102,6 +33648,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U311" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
@@ -32204,6 +33755,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U312" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
@@ -32306,6 +33862,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U313" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
@@ -32408,6 +33969,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U314" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
@@ -32510,6 +34076,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U315" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
@@ -32612,6 +34183,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U316" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
@@ -32714,6 +34290,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U317" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
@@ -32816,6 +34397,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U318" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
@@ -32918,6 +34504,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U319" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
@@ -33020,6 +34611,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U320" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
@@ -33122,6 +34718,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U321" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="4" t="inlineStr">
@@ -33224,6 +34825,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U322" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
@@ -33326,6 +34932,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U323" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
@@ -33428,6 +35039,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U324" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
@@ -33530,6 +35146,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U325" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
@@ -33632,6 +35253,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U326" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
@@ -33734,6 +35360,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U327" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
@@ -33836,6 +35467,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U328" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
@@ -33938,6 +35574,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U329" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
@@ -34040,6 +35681,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U330" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
@@ -34142,6 +35788,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U331" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
@@ -34244,6 +35895,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U332" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
@@ -34346,6 +36002,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U333" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
@@ -34448,6 +36109,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U334" s="4" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
@@ -34550,6 +36216,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U335" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="4" t="inlineStr">
@@ -34652,6 +36323,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U336" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
@@ -34754,6 +36430,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U337" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="4" t="inlineStr">
@@ -34856,6 +36537,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U338" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="4" t="inlineStr">
@@ -34958,6 +36644,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U339" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="4" t="inlineStr">
@@ -35060,6 +36751,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U340" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="4" t="inlineStr">
@@ -35162,6 +36858,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U341" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="4" t="inlineStr">
@@ -35264,6 +36965,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U342" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="4" t="inlineStr">
@@ -35366,6 +37072,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U343" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="4" t="inlineStr">
@@ -35468,6 +37179,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U344" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="4" t="inlineStr">
@@ -35570,6 +37286,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U345" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="4" t="inlineStr">
@@ -35672,6 +37393,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U346" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="4" t="inlineStr">
@@ -35774,6 +37500,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U347" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="4" t="inlineStr">
@@ -35876,6 +37607,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U348" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="4" t="inlineStr">
@@ -35978,6 +37714,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U349" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="4" t="inlineStr">
@@ -36080,6 +37821,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U350" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="4" t="inlineStr">
@@ -36182,6 +37928,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U351" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="4" t="inlineStr">
@@ -36284,6 +38035,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U352" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="4" t="inlineStr">
@@ -36386,6 +38142,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U353" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="4" t="inlineStr">
@@ -36488,6 +38249,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U354" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="4" t="inlineStr">
@@ -36590,6 +38356,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U355" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="4" t="inlineStr">
@@ -36692,6 +38463,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U356" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="4" t="inlineStr">
@@ -36794,6 +38570,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U357" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="4" t="inlineStr">
@@ -36896,6 +38677,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U358" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="4" t="inlineStr">
@@ -36998,6 +38784,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U359" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="4" t="inlineStr">
@@ -37100,6 +38891,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U360" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="4" t="inlineStr">
@@ -37202,6 +38998,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U361" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="4" t="inlineStr">
@@ -37304,6 +39105,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U362" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="4" t="inlineStr">
@@ -37406,6 +39212,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U363" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="4" t="inlineStr">
@@ -37508,6 +39319,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U364" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="4" t="inlineStr">
@@ -37610,6 +39426,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U365" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="4" t="inlineStr">
@@ -37712,6 +39533,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U366" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="4" t="inlineStr">
@@ -37814,6 +39640,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U367" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="4" t="inlineStr">
@@ -37916,6 +39747,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U368" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="4" t="inlineStr">
@@ -38018,6 +39854,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U369" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="4" t="inlineStr">
@@ -38120,6 +39961,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U370" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="4" t="inlineStr">
@@ -38222,6 +40068,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U371" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="4" t="inlineStr">
@@ -38324,6 +40175,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U372" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="4" t="inlineStr">
@@ -38426,6 +40282,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U373" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="4" t="inlineStr">
@@ -38528,6 +40389,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U374" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="4" t="inlineStr">
@@ -38630,6 +40496,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U375" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="4" t="inlineStr">
@@ -38732,6 +40603,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U376" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="4" t="inlineStr">
@@ -38834,6 +40710,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U377" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="4" t="inlineStr">
@@ -38936,6 +40817,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U378" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="4" t="inlineStr">
@@ -39038,6 +40924,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U379" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="4" t="inlineStr">
@@ -39140,6 +41031,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U380" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="4" t="inlineStr">
@@ -39242,6 +41138,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U381" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="4" t="inlineStr">
@@ -39344,6 +41245,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U382" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="4" t="inlineStr">
@@ -39446,6 +41352,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U383" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="4" t="inlineStr">
@@ -39548,6 +41459,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U384" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="4" t="inlineStr">
@@ -39650,6 +41566,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U385" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="4" t="inlineStr">
@@ -39752,6 +41673,11 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U386" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="4" t="inlineStr">
@@ -39854,11 +41780,16 @@
           <t>40615</t>
         </is>
       </c>
+      <c r="U387" s="4" t="inlineStr">
+        <is>
+          <t>WARGA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:T387"/>
+  <autoFilter ref="A2:U387"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A1:U1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: pilihan peran di halaman masuk, menu Ganti Password, JWT_SECRET wajib diisi
Halaman masuk menampilkan empat peran beserta contoh username tiap peran.
Pilihannya TIDAK dikirim ke backend dan tidak menentukan apa pun: peran melekat
pada akun, dan memaksakannya cocok justru memberi tahu penebak password peran
apa yang dipegang sebuah username.

Menu Ganti Password ditambahkan ke dropdown akun — sebelumnya halamannya ada
tapi cuma bisa dicapai dengan mengetik alamatnya sendiri.

JWT_SECRET bawaan sekarang menolak jalan, sama tegas dengan ADMIN_PASSWORD.
Defaultnya tetap ada supaya perkakas baris perintah jalan tanpa .env.

Kolom Jabatan di docs/data-penduduk.xlsx disetel WARGA semua.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data-penduduk.xlsx
+++ b/docs/data-penduduk.xlsx
@@ -2192,7 +2192,7 @@
       </c>
       <c r="U17" s="4" t="inlineStr">
         <is>
-          <t>DUKUH</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>
@@ -11073,7 +11073,7 @@
       </c>
       <c r="U100" s="4" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>
@@ -17600,7 +17600,7 @@
       </c>
       <c r="U161" s="4" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>
@@ -20810,7 +20810,7 @@
       </c>
       <c r="U191" s="4" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>
@@ -26802,7 +26802,7 @@
       </c>
       <c r="U247" s="4" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>
@@ -27123,7 +27123,7 @@
       </c>
       <c r="U250" s="4" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>
@@ -27872,7 +27872,7 @@
       </c>
       <c r="U257" s="4" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>
@@ -28942,7 +28942,7 @@
       </c>
       <c r="U267" s="4" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>
@@ -30868,7 +30868,7 @@
       </c>
       <c r="U285" s="4" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>
@@ -36111,7 +36111,7 @@
       </c>
       <c r="U334" s="4" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>WARGA</t>
         </is>
       </c>
     </row>

</xml_diff>